<commit_message>
add: Cambio de nombre en FiliterListDto de Asientos
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/Venta Impuestos.xlsx
+++ b/api/src/main/resources/importaciones/Venta Impuestos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8998CE32-C804-4E7A-AADA-7BDED1E26DC9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92273CD0-02B1-4737-8D1A-E080DDC4A2BB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{6E3A5EA0-8E38-4FC7-96C7-04052A5F8F56}"/>
   </bookViews>
@@ -340,6 +340,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -379,10 +382,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,6 +705,7 @@
   <cols>
     <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="20.85546875" customWidth="1"/>
+    <col min="11" max="11" width="23" style="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
@@ -735,7 +739,7 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="7" t="s">
         <v>10</v>
       </c>
       <c r="L1" t="s">
@@ -800,7 +804,7 @@
       <c r="J2" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="4">
+      <c r="K2" s="7">
         <v>46143</v>
       </c>
       <c r="L2">
@@ -824,7 +828,7 @@
       <c r="T2">
         <v>0</v>
       </c>
-      <c r="U2" s="5" t="s">
+      <c r="U2" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -859,7 +863,7 @@
       <c r="J3" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="4">
+      <c r="K3" s="7">
         <v>46143</v>
       </c>
       <c r="L3">
@@ -877,7 +881,7 @@
       <c r="T3">
         <v>0</v>
       </c>
-      <c r="U3" s="5" t="s">
+      <c r="U3" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -912,7 +916,7 @@
       <c r="J4" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="7">
         <v>46143</v>
       </c>
       <c r="L4">
@@ -930,7 +934,7 @@
       <c r="T4">
         <v>0</v>
       </c>
-      <c r="U4" s="5" t="s">
+      <c r="U4" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -965,7 +969,7 @@
       <c r="J5" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="7">
         <v>46143</v>
       </c>
       <c r="L5">
@@ -983,7 +987,7 @@
       <c r="T5">
         <v>0</v>
       </c>
-      <c r="U5" s="5" t="s">
+      <c r="U5" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1018,7 +1022,7 @@
       <c r="J6" t="s">
         <v>28</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="7">
         <v>46143</v>
       </c>
       <c r="L6">
@@ -1036,7 +1040,7 @@
       <c r="T6">
         <v>0</v>
       </c>
-      <c r="U6" s="5" t="s">
+      <c r="U6" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1071,7 +1075,7 @@
       <c r="J7" t="s">
         <v>28</v>
       </c>
-      <c r="K7" s="4">
+      <c r="K7" s="7">
         <v>46143</v>
       </c>
       <c r="L7">
@@ -1089,7 +1093,7 @@
       <c r="T7">
         <v>0</v>
       </c>
-      <c r="U7" s="5" t="s">
+      <c r="U7" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1124,7 +1128,7 @@
       <c r="J8" t="s">
         <v>28</v>
       </c>
-      <c r="K8" s="4">
+      <c r="K8" s="7">
         <v>46143</v>
       </c>
       <c r="L8">
@@ -1142,7 +1146,7 @@
       <c r="T8">
         <v>0</v>
       </c>
-      <c r="U8" s="5" t="s">
+      <c r="U8" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1177,7 +1181,7 @@
       <c r="J9" t="s">
         <v>28</v>
       </c>
-      <c r="K9" s="4">
+      <c r="K9" s="7">
         <v>46143</v>
       </c>
       <c r="L9">
@@ -1195,7 +1199,7 @@
       <c r="T9">
         <v>0</v>
       </c>
-      <c r="U9" s="5" t="s">
+      <c r="U9" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1230,7 +1234,7 @@
       <c r="J10" t="s">
         <v>28</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="7">
         <v>46143</v>
       </c>
       <c r="L10">
@@ -1248,7 +1252,7 @@
       <c r="T10">
         <v>0</v>
       </c>
-      <c r="U10" s="5" t="s">
+      <c r="U10" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1283,7 +1287,7 @@
       <c r="J11" t="s">
         <v>28</v>
       </c>
-      <c r="K11" s="4">
+      <c r="K11" s="7">
         <v>46143</v>
       </c>
       <c r="L11">
@@ -1301,7 +1305,7 @@
       <c r="T11">
         <v>0</v>
       </c>
-      <c r="U11" s="5" t="s">
+      <c r="U11" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1336,7 +1340,7 @@
       <c r="J12" t="s">
         <v>28</v>
       </c>
-      <c r="K12" s="4">
+      <c r="K12" s="7">
         <v>46143</v>
       </c>
       <c r="L12">
@@ -1354,7 +1358,7 @@
       <c r="T12">
         <v>0</v>
       </c>
-      <c r="U12" s="5" t="s">
+      <c r="U12" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1389,7 +1393,7 @@
       <c r="J13" t="s">
         <v>28</v>
       </c>
-      <c r="K13" s="4">
+      <c r="K13" s="7">
         <v>46143</v>
       </c>
       <c r="L13">
@@ -1407,7 +1411,7 @@
       <c r="T13">
         <v>0</v>
       </c>
-      <c r="U13" s="5" t="s">
+      <c r="U13" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1442,7 +1446,7 @@
       <c r="J14" t="s">
         <v>28</v>
       </c>
-      <c r="K14" s="4">
+      <c r="K14" s="7">
         <v>46143</v>
       </c>
       <c r="L14">
@@ -1460,7 +1464,7 @@
       <c r="T14">
         <v>0</v>
       </c>
-      <c r="U14" s="5" t="s">
+      <c r="U14" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1495,7 +1499,7 @@
       <c r="J15" t="s">
         <v>28</v>
       </c>
-      <c r="K15" s="4">
+      <c r="K15" s="7">
         <v>46143</v>
       </c>
       <c r="L15">
@@ -1513,7 +1517,7 @@
       <c r="T15">
         <v>0</v>
       </c>
-      <c r="U15" s="5" t="s">
+      <c r="U15" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1548,7 +1552,7 @@
       <c r="J16" t="s">
         <v>28</v>
       </c>
-      <c r="K16" s="4">
+      <c r="K16" s="7">
         <v>46143</v>
       </c>
       <c r="L16">
@@ -1566,7 +1570,7 @@
       <c r="T16">
         <v>0</v>
       </c>
-      <c r="U16" s="5" t="s">
+      <c r="U16" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1601,7 +1605,7 @@
       <c r="J17" t="s">
         <v>28</v>
       </c>
-      <c r="K17" s="4">
+      <c r="K17" s="7">
         <v>46143</v>
       </c>
       <c r="L17">
@@ -1619,7 +1623,7 @@
       <c r="T17">
         <v>0</v>
       </c>
-      <c r="U17" s="5" t="s">
+      <c r="U17" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1654,7 +1658,7 @@
       <c r="J18" t="s">
         <v>28</v>
       </c>
-      <c r="K18" s="4">
+      <c r="K18" s="7">
         <v>46143</v>
       </c>
       <c r="L18">
@@ -1672,7 +1676,7 @@
       <c r="T18">
         <v>0</v>
       </c>
-      <c r="U18" s="5" t="s">
+      <c r="U18" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1707,7 +1711,7 @@
       <c r="J19" t="s">
         <v>28</v>
       </c>
-      <c r="K19" s="4">
+      <c r="K19" s="7">
         <v>46143</v>
       </c>
       <c r="L19">
@@ -1725,7 +1729,7 @@
       <c r="T19">
         <v>0</v>
       </c>
-      <c r="U19" s="5" t="s">
+      <c r="U19" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1760,7 +1764,7 @@
       <c r="J20" t="s">
         <v>28</v>
       </c>
-      <c r="K20" s="4">
+      <c r="K20" s="7">
         <v>46143</v>
       </c>
       <c r="L20">
@@ -1778,7 +1782,7 @@
       <c r="T20">
         <v>0</v>
       </c>
-      <c r="U20" s="5" t="s">
+      <c r="U20" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1813,7 +1817,7 @@
       <c r="J21" t="s">
         <v>28</v>
       </c>
-      <c r="K21" s="4">
+      <c r="K21" s="7">
         <v>46143</v>
       </c>
       <c r="L21">
@@ -1831,7 +1835,7 @@
       <c r="T21">
         <v>0</v>
       </c>
-      <c r="U21" s="5" t="s">
+      <c r="U21" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1866,7 +1870,7 @@
       <c r="J22" t="s">
         <v>28</v>
       </c>
-      <c r="K22" s="4">
+      <c r="K22" s="7">
         <v>46143</v>
       </c>
       <c r="L22">
@@ -1884,7 +1888,7 @@
       <c r="T22">
         <v>0</v>
       </c>
-      <c r="U22" s="5" t="s">
+      <c r="U22" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1919,7 +1923,7 @@
       <c r="J23" t="s">
         <v>28</v>
       </c>
-      <c r="K23" s="4">
+      <c r="K23" s="7">
         <v>46143</v>
       </c>
       <c r="L23">
@@ -1937,7 +1941,7 @@
       <c r="T23">
         <v>0</v>
       </c>
-      <c r="U23" s="5" t="s">
+      <c r="U23" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1972,7 +1976,7 @@
       <c r="J24" t="s">
         <v>28</v>
       </c>
-      <c r="K24" s="4">
+      <c r="K24" s="7">
         <v>46143</v>
       </c>
       <c r="L24">
@@ -1990,7 +1994,7 @@
       <c r="T24">
         <v>0</v>
       </c>
-      <c r="U24" s="5" t="s">
+      <c r="U24" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2025,7 +2029,7 @@
       <c r="J25" t="s">
         <v>28</v>
       </c>
-      <c r="K25" s="4">
+      <c r="K25" s="7">
         <v>46143</v>
       </c>
       <c r="L25">
@@ -2043,7 +2047,7 @@
       <c r="T25">
         <v>0</v>
       </c>
-      <c r="U25" s="5" t="s">
+      <c r="U25" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2078,7 +2082,7 @@
       <c r="J26" t="s">
         <v>28</v>
       </c>
-      <c r="K26" s="4">
+      <c r="K26" s="7">
         <v>46143</v>
       </c>
       <c r="L26">
@@ -2096,7 +2100,7 @@
       <c r="T26">
         <v>0</v>
       </c>
-      <c r="U26" s="5" t="s">
+      <c r="U26" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2131,7 +2135,7 @@
       <c r="J27" t="s">
         <v>28</v>
       </c>
-      <c r="K27" s="4">
+      <c r="K27" s="7">
         <v>46143</v>
       </c>
       <c r="L27">
@@ -2149,7 +2153,7 @@
       <c r="T27">
         <v>0</v>
       </c>
-      <c r="U27" s="5" t="s">
+      <c r="U27" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2184,7 +2188,7 @@
       <c r="J28" t="s">
         <v>28</v>
       </c>
-      <c r="K28" s="4">
+      <c r="K28" s="7">
         <v>46143</v>
       </c>
       <c r="L28">
@@ -2202,7 +2206,7 @@
       <c r="T28">
         <v>0</v>
       </c>
-      <c r="U28" s="5" t="s">
+      <c r="U28" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2237,7 +2241,7 @@
       <c r="J29" t="s">
         <v>28</v>
       </c>
-      <c r="K29" s="4">
+      <c r="K29" s="7">
         <v>46143</v>
       </c>
       <c r="L29">
@@ -2255,7 +2259,7 @@
       <c r="T29">
         <v>0</v>
       </c>
-      <c r="U29" s="5" t="s">
+      <c r="U29" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2290,7 +2294,7 @@
       <c r="J30" t="s">
         <v>28</v>
       </c>
-      <c r="K30" s="4">
+      <c r="K30" s="7">
         <v>46143</v>
       </c>
       <c r="L30">
@@ -2308,7 +2312,7 @@
       <c r="T30">
         <v>0</v>
       </c>
-      <c r="U30" s="5" t="s">
+      <c r="U30" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2343,7 +2347,7 @@
       <c r="J31" t="s">
         <v>28</v>
       </c>
-      <c r="K31" s="4">
+      <c r="K31" s="7">
         <v>46143</v>
       </c>
       <c r="L31">
@@ -2361,7 +2365,7 @@
       <c r="T31">
         <v>0</v>
       </c>
-      <c r="U31" s="5" t="s">
+      <c r="U31" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2396,7 +2400,7 @@
       <c r="J32" t="s">
         <v>28</v>
       </c>
-      <c r="K32" s="4">
+      <c r="K32" s="7">
         <v>46143</v>
       </c>
       <c r="L32">
@@ -2414,7 +2418,7 @@
       <c r="T32">
         <v>0</v>
       </c>
-      <c r="U32" s="5" t="s">
+      <c r="U32" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2449,7 +2453,7 @@
       <c r="J33" t="s">
         <v>28</v>
       </c>
-      <c r="K33" s="4">
+      <c r="K33" s="7">
         <v>46143</v>
       </c>
       <c r="L33">
@@ -2467,7 +2471,7 @@
       <c r="T33">
         <v>0</v>
       </c>
-      <c r="U33" s="5" t="s">
+      <c r="U33" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2502,7 +2506,7 @@
       <c r="J34" t="s">
         <v>28</v>
       </c>
-      <c r="K34" s="4">
+      <c r="K34" s="7">
         <v>46143</v>
       </c>
       <c r="L34">
@@ -2520,7 +2524,7 @@
       <c r="T34">
         <v>0</v>
       </c>
-      <c r="U34" s="5" t="s">
+      <c r="U34" s="4" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2540,7 +2544,7 @@
       <c r="E35" t="s">
         <v>25</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="F35" s="5" t="s">
         <v>99</v>
       </c>
       <c r="G35" t="s">
@@ -2552,10 +2556,10 @@
       <c r="I35" t="s">
         <v>28</v>
       </c>
-      <c r="J35" s="7" t="s">
+      <c r="J35" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="K35" s="4">
+      <c r="K35" s="7">
         <v>46143</v>
       </c>
       <c r="L35">
@@ -2573,7 +2577,7 @@
       <c r="T35">
         <v>0</v>
       </c>
-      <c r="U35" s="5" t="s">
+      <c r="U35" s="4" t="s">
         <v>102</v>
       </c>
     </row>

</xml_diff>